<commit_message>
connect tc_6(new payment related fix)
</commit_message>
<xml_diff>
--- a/test_data/make_payment.xlsx
+++ b/test_data/make_payment.xlsx
@@ -470,25 +470,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>75c44810a32a3d6447df</t>
+          <t>7bd45c59c31792c2cb70</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>+74267426016</t>
+          <t>+74267426055</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Automation User 10</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>100</v>
+          <t>Automation User 55</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fixes for opportunity creation web test case
</commit_message>
<xml_diff>
--- a/test_data/make_payment.xlsx
+++ b/test_data/make_payment.xlsx
@@ -470,25 +470,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>75c44810a32a3d6447df</t>
+          <t>7bd45c59c31792c2cb70</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>+74267426016</t>
+          <t>+74267426055</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Automation User 10</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>100</v>
+          <t>Automation User 55</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-05-12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fixes for new web login UI change
</commit_message>
<xml_diff>
--- a/test_data/make_payment.xlsx
+++ b/test_data/make_payment.xlsx
@@ -470,27 +470,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>7bd45c59c31792c2cb70</t>
+          <t>75c44810a32a3d6447df</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>+74267426055</t>
+          <t>+74267426016</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Automation User 55</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
+          <t>Automation User 10</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>100</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fixes for prod web and mobile(seperated payment test) tests
</commit_message>
<xml_diff>
--- a/test_data/make_payment.xlsx
+++ b/test_data/make_payment.xlsx
@@ -470,25 +470,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>75c44810a32a3d6447df</t>
+          <t>3c51eef69294b8826412</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>+74267426016</t>
+          <t>+74267426017</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Automation User 10</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>100</v>
+          <t>Automation User 17</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>431</t>
+        </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
new changes to mobile test_6
</commit_message>
<xml_diff>
--- a/test_data/make_payment.xlsx
+++ b/test_data/make_payment.xlsx
@@ -485,12 +485,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>431</t>
+          <t>94</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
apk changed to 2.63 version
</commit_message>
<xml_diff>
--- a/test_data/make_payment.xlsx
+++ b/test_data/make_payment.xlsx
@@ -485,12 +485,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>94</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>

</xml_diff>